<commit_message>
Add NRV live URL and a Live field in the project content template.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/portfolio/nrv-web/NRV - WEB.xlsx
+++ b/public/portfolio/nrv-web/NRV - WEB.xlsx
@@ -12,17 +12,38 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="130">
+  <si>
+    <t>Block</t>
+  </si>
   <si>
     <t>How to fill</t>
   </si>
   <si>
-    <t>Block</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
+    <t>1. Fill columns PL / EN / ES for each field.</t>
+  </si>
+  <si>
+    <t>2. Section 1-10 map to case-study sections (max 10). Leave unused sections empty.</t>
+  </si>
+  <si>
+    <t>3. Label = sidebar name (e.g. OVERVIEW, WYZWANIA, RESULTS).</t>
+  </si>
+  <si>
+    <t>4. Title = section heading. Description = body copy.</t>
+  </si>
+  <si>
+    <t>5. Hero Title = project hero headline.</t>
+  </si>
+  <si>
+    <t>6. Meta: Services, Industry, Market, Year.</t>
+  </si>
+  <si>
+    <t>7. One sheet = one project. Duplicate "Project translations" for more projects.</t>
+  </si>
+  <si>
     <t>Field</t>
   </si>
   <si>
@@ -38,27 +59,6 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>1. Fill columns PL / EN / ES for each field.</t>
-  </si>
-  <si>
-    <t>2. Section 1-10 map to case-study sections (max 10). Leave unused sections empty.</t>
-  </si>
-  <si>
-    <t>3. Label = sidebar name (e.g. OVERVIEW, WYZWANIA, RESULTS).</t>
-  </si>
-  <si>
-    <t>4. Title = section heading. Description = body copy.</t>
-  </si>
-  <si>
-    <t>5. Hero Title = project hero headline.</t>
-  </si>
-  <si>
-    <t>6. Meta: Services, Industry, Market, Year.</t>
-  </si>
-  <si>
-    <t>7. One sheet = one project. Duplicate "Project translations" for more projects.</t>
-  </si>
-  <si>
     <t>Project</t>
   </si>
   <si>
@@ -128,22 +128,28 @@
     <t>Rok / Year / Año</t>
   </si>
   <si>
-    <t>np. 2024</t>
+    <t>np. 2023</t>
+  </si>
+  <si>
+    <t>Live</t>
+  </si>
+  <si>
+    <t>nrvsystems.com</t>
+  </si>
+  <si>
+    <t>https://www.nrvsystems.com/</t>
   </si>
   <si>
     <t>Section 1</t>
   </si>
   <si>
-    <t>Label</t>
+    <t>Contexto</t>
   </si>
   <si>
     <t>Kontekst</t>
   </si>
   <si>
     <t>Overview</t>
-  </si>
-  <si>
-    <t>Contexto</t>
   </si>
   <si>
     <t>np. Overview / Intro</t>
@@ -180,6 +186,9 @@
   </si>
   <si>
     <t>Section 2</t>
+  </si>
+  <si>
+    <t>Label</t>
   </si>
   <si>
     <t>Audyt i Badania</t>
@@ -423,7 +432,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -437,19 +446,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11.0"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -523,15 +538,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="2" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
@@ -559,14 +574,20 @@
     <xf borderId="2" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
+    <xf borderId="2" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="6" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
@@ -806,44 +827,44 @@
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="T1" s="3"/>
+      <c r="U1" s="3"/>
+      <c r="V1" s="3"/>
+      <c r="W1" s="3"/>
+      <c r="X1" s="3"/>
+      <c r="Y1" s="3"/>
+      <c r="Z1" s="3"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="s">
@@ -966,7 +987,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="13" t="s">
         <v>26</v>
       </c>
       <c r="B8" s="11" t="s">
@@ -986,606 +1007,622 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="D9" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="D9" s="15" t="s">
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="B10" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="14" t="s">
+      <c r="C10" s="16" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" s="14" t="s">
+      <c r="D10" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="F10" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="15" t="s">
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F10" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" ht="60.0" customHeight="1">
-      <c r="A11" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" s="14" t="s">
+      <c r="D11" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="E11" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="F11" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" ht="60.0" customHeight="1">
+      <c r="A12" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="D12" s="16" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="16" t="s">
+      <c r="E12" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="18" t="s">
+      <c r="F12" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="18" t="s">
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F13" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" ht="60.0" customHeight="1">
-      <c r="A14" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="18" t="s">
+      <c r="F13" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="s">
+      <c r="F14" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="60.0" customHeight="1">
+      <c r="A15" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="15" t="s">
+      <c r="D15" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="E15" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="F15" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="15" t="s">
+      <c r="B16" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" ht="60.0" customHeight="1">
-      <c r="A17" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="15" t="s">
+      <c r="F16" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E17" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="F17" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="16" t="s">
+      <c r="F17" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" ht="60.0" customHeight="1">
+      <c r="A18" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="F18" s="17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="F18" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="18" t="s">
+      <c r="B19" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" ht="60.0" customHeight="1">
-      <c r="A20" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C20" s="18" t="s">
+      <c r="F19" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="E20" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="F20" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="13" t="s">
+      <c r="F20" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" ht="60.0" customHeight="1">
+      <c r="A21" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="B21" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="15" t="s">
+      <c r="D21" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="E21" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="F21" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="F21" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="15" t="s">
+      <c r="B22" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="F22" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" ht="60.0" customHeight="1">
-      <c r="A23" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C23" s="15" t="s">
+      <c r="F22" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="16" t="s">
+      <c r="F23" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" ht="60.0" customHeight="1">
+      <c r="A24" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="18" t="s">
+      <c r="D24" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="F24" s="17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="F24" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="18" t="s">
+      <c r="B25" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="E25" s="18" t="s">
+      <c r="E25" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="F25" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" ht="60.0" customHeight="1">
-      <c r="A26" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C26" s="18" t="s">
+      <c r="F25" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="D26" s="18" t="s">
+      <c r="D26" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="E26" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="13" t="s">
+      <c r="F26" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" ht="60.0" customHeight="1">
+      <c r="A27" s="18" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C27" s="15" t="s">
+      <c r="D27" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="15" t="s">
+      <c r="E27" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="E27" s="15" t="s">
+      <c r="F27" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="15" t="s">
         <v>107</v>
       </c>
-      <c r="F27" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28" s="15" t="s">
+      <c r="B28" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C28" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="F28" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" ht="60.0" customHeight="1">
-      <c r="A29" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C29" s="15" t="s">
+      <c r="F28" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="16" t="s">
         <v>113</v>
       </c>
-      <c r="F29" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="16" t="s">
+      <c r="F29" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" ht="60.0" customHeight="1">
+      <c r="A30" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="C30" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="B30" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D30" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="E30" s="17" t="s">
-        <v>2</v>
+      <c r="D30" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>116</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>2</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B31" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D31" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="F31" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" ht="60.0" customHeight="1">
-      <c r="A32" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C32" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="D32" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B33" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D33" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="F33" s="14" t="s">
-        <v>2</v>
+      <c r="A31" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="F32" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" ht="60.0" customHeight="1">
+      <c r="A33" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B34" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="F34" s="14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" ht="60.0" customHeight="1">
-      <c r="A35" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="E35" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="F35" s="14" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="16" t="s">
-        <v>116</v>
+      <c r="A34" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" ht="60.0" customHeight="1">
+      <c r="A36" s="15" t="s">
+        <v>118</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>117</v>
-      </c>
-      <c r="D36" s="18" t="s">
-        <v>118</v>
-      </c>
-      <c r="E36" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="18" t="s">
         <v>119</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="B37" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="20" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B37" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="C37" s="18" t="s">
+      <c r="D37" s="20" t="s">
         <v>121</v>
       </c>
-      <c r="D37" s="18" t="s">
+      <c r="E37" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="18" t="s">
+      <c r="F37" s="19" t="s">
         <v>123</v>
       </c>
-      <c r="F37" s="17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" ht="60.0" customHeight="1">
-      <c r="A38" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="18" t="s">
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C38" s="20" t="s">
         <v>124</v>
       </c>
-      <c r="D38" s="18" t="s">
+      <c r="D38" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="E38" s="18" t="s">
+      <c r="E38" s="20" t="s">
         <v>126</v>
       </c>
-      <c r="F38" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1"/>
+      <c r="F38" s="19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" ht="60.0" customHeight="1">
+      <c r="A39" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="D39" s="20" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" s="20" t="s">
+        <v>129</v>
+      </c>
+      <c r="F39" s="19" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="40" ht="15.75" customHeight="1"/>
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -2547,11 +2584,18 @@
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="C9"/>
+    <hyperlink r:id="rId2" ref="D9"/>
+    <hyperlink r:id="rId3" ref="E9"/>
+    <hyperlink r:id="rId4" ref="F9"/>
+  </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -2568,7 +2612,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2597,43 +2641,43 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="9">
+      <c r="A9" s="2" t="s">
         <v>9</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>